<commit_message>
v1.10.4 SINGLE FORMAT: Items + Opening Stock qty/rate/date/narration in ONE Excel, no secondary system
- ITEM_COLS now name,unit,hsn,gst_rate,is_service,sale_account,purchase_account,qty,rate,date,narration
- importKind items: collects qty/rate/date/narration per row, groups by date, auto-finds counterpart (Opening Stock / Reserves & Surplus / Capital or creates adjustment), creates Stock Journal vouchers per date inside same tx for buy vs sell age tracking
- ItemExcel.jsx: MAP 11 cols, header single format with stock+date, no secondary mentions
- Masters.jsx ItemsTab: only ItemExcelPanel, StockExcelPanel deleted
- Data.jsx: removed stock kind entirely, only ledgers/items/vouchers, items tip says SINGLE FORMAT no second file
- templates regenerated, sample file now includes qty/rate/date/narration
- dist included in zip, batch %~dp0. fix for space in path, build fallback

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/templates/template-2-stock-items.xlsx
+++ b/templates/template-2-stock-items.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:K2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,6 +422,18 @@
       <c r="G1" t="str">
         <v>purchase_account</v>
       </c>
+      <c r="H1" t="str">
+        <v>qty</v>
+      </c>
+      <c r="I1" t="str">
+        <v>rate</v>
+      </c>
+      <c r="J1" t="str">
+        <v>date</v>
+      </c>
+      <c r="K1" t="str">
+        <v>narration</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -445,29 +457,51 @@
       <c r="G2" t="str">
         <v/>
       </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A3"/>
   <cols>
     <col min="1" max="1" width="110.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Fill one item per row. Required: name. Example row is marked EXAMPLE — delete it before importing.</v>
+        <v>SINGLE FORMAT: one row per item — master + opening stock + date in SAME file. Required: name.</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>If you fill qty+rate in same row, stock is auto-added with that date for buy vs sell age tracking.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Optional: qty, rate, date (YYYY-MM-DD), narration (batch/supplier). Example row is marked EXAMPLE — delete it before importing.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>